<commit_message>
J4 merged with Control Board BOM
</commit_message>
<xml_diff>
--- a/Deliverables/Control_Board/BOM/Control_Board_BOM (500 Boards).xlsx
+++ b/Deliverables/Control_Board/BOM/Control_Board_BOM (500 Boards).xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25330"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\ChristianRaun-EthercatDesign\Deliverables\Control_Board\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Faizan\GitHub\ChristianRaun-EthercatDesign\Deliverables\Control_Board\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{370284ED-8F79-40EB-8105-287A2A756DD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -30,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="189">
   <si>
     <t>Component list</t>
   </si>
@@ -589,9 +588,6 @@
     <t>---------</t>
   </si>
   <si>
-    <t xml:space="preserve">1x40 pins Header 5 PCS per Lot </t>
-  </si>
-  <si>
     <t>Custom Supplier</t>
   </si>
   <si>
@@ -599,12 +595,18 @@
   </si>
   <si>
     <t>Already Purchas From Client Side</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 x 30 pins Header 10 PCS per Lot </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 x 40 pins Header 10 PCS per Lot </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0000"/>
@@ -1485,6 +1487,15 @@
     <xf numFmtId="165" fontId="18" fillId="2" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="18" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="27" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="27" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
@@ -1559,15 +1570,6 @@
     <xf numFmtId="0" fontId="27" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="4" borderId="18" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="27" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1613,7 +1615,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1909,7 +1911,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:S39"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1945,15 +1947,15 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="116"/>
-      <c r="L1" s="116"/>
-      <c r="M1" s="116"/>
-      <c r="N1" s="116"/>
-      <c r="O1" s="116"/>
-      <c r="P1" s="116"/>
-      <c r="Q1" s="116"/>
-      <c r="R1" s="116"/>
-      <c r="S1" s="117"/>
+      <c r="K1" s="119"/>
+      <c r="L1" s="119"/>
+      <c r="M1" s="119"/>
+      <c r="N1" s="119"/>
+      <c r="O1" s="119"/>
+      <c r="P1" s="119"/>
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="120"/>
     </row>
     <row r="2" spans="1:19" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -2003,7 +2005,7 @@
       <c r="P3" s="5"/>
       <c r="Q3" s="5"/>
       <c r="R3" s="5"/>
-      <c r="S3" s="118"/>
+      <c r="S3" s="121"/>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -2028,7 +2030,7 @@
       <c r="P4" s="6"/>
       <c r="Q4" s="6"/>
       <c r="R4" s="6"/>
-      <c r="S4" s="119"/>
+      <c r="S4" s="122"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -2053,7 +2055,7 @@
       <c r="P5" s="6"/>
       <c r="Q5" s="6"/>
       <c r="R5" s="6"/>
-      <c r="S5" s="119"/>
+      <c r="S5" s="122"/>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -2074,7 +2076,7 @@
       <c r="P6" s="6"/>
       <c r="Q6" s="6"/>
       <c r="R6" s="6"/>
-      <c r="S6" s="119"/>
+      <c r="S6" s="122"/>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -2095,7 +2097,7 @@
       <c r="P7" s="8"/>
       <c r="Q7" s="8"/>
       <c r="R7" s="8"/>
-      <c r="S7" s="119"/>
+      <c r="S7" s="122"/>
     </row>
     <row r="8" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -2116,7 +2118,7 @@
       <c r="P8" s="8"/>
       <c r="Q8" s="8"/>
       <c r="R8" s="8"/>
-      <c r="S8" s="119"/>
+      <c r="S8" s="122"/>
     </row>
     <row r="9" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -2181,7 +2183,7 @@
         <f>ROW(B10) - ROW($B$9)</f>
         <v>1</v>
       </c>
-      <c r="C10" s="124" t="s">
+      <c r="C10" s="127" t="s">
         <v>151</v>
       </c>
       <c r="D10" s="43" t="s">
@@ -2237,7 +2239,7 @@
         <f t="shared" ref="B11:B35" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
-      <c r="C11" s="125"/>
+      <c r="C11" s="128"/>
       <c r="D11" s="47" t="s">
         <v>12</v>
       </c>
@@ -2291,7 +2293,7 @@
         <f>ROW(B12) - ROW($B$9)</f>
         <v>3</v>
       </c>
-      <c r="C12" s="125"/>
+      <c r="C12" s="128"/>
       <c r="D12" s="43" t="s">
         <v>13</v>
       </c>
@@ -2345,7 +2347,7 @@
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="125"/>
+      <c r="C13" s="128"/>
       <c r="D13" s="47" t="s">
         <v>14</v>
       </c>
@@ -2399,7 +2401,7 @@
         <f>ROW(B14) - ROW($B$9)</f>
         <v>5</v>
       </c>
-      <c r="C14" s="125"/>
+      <c r="C14" s="128"/>
       <c r="D14" s="43" t="s">
         <v>15</v>
       </c>
@@ -2453,7 +2455,7 @@
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C15" s="124" t="s">
+      <c r="C15" s="127" t="s">
         <v>152</v>
       </c>
       <c r="D15" s="47" t="s">
@@ -2487,21 +2489,21 @@
         <f t="shared" si="1"/>
         <v>500</v>
       </c>
-      <c r="N15" s="114">
-        <v>140</v>
-      </c>
-      <c r="O15" s="127" t="s">
+      <c r="N15" s="117">
+        <v>17</v>
+      </c>
+      <c r="O15" s="130" t="s">
         <v>175</v>
       </c>
-      <c r="P15" s="110">
-        <v>0.41</v>
-      </c>
-      <c r="Q15" s="112">
+      <c r="P15" s="113">
+        <v>4.9411764705882302</v>
+      </c>
+      <c r="Q15" s="115">
         <f t="shared" si="2"/>
-        <v>57.4</v>
-      </c>
-      <c r="R15" s="108" t="s">
-        <v>184</v>
+        <v>83.999999999999915</v>
+      </c>
+      <c r="R15" s="111" t="s">
+        <v>188</v>
       </c>
       <c r="S15" s="51"/>
     </row>
@@ -2511,7 +2513,7 @@
         <f>ROW(B16) - ROW($B$9)</f>
         <v>7</v>
       </c>
-      <c r="C16" s="125"/>
+      <c r="C16" s="128"/>
       <c r="D16" s="43" t="s">
         <v>17</v>
       </c>
@@ -2543,11 +2545,11 @@
         <f t="shared" si="1"/>
         <v>500</v>
       </c>
-      <c r="N16" s="115"/>
-      <c r="O16" s="128"/>
-      <c r="P16" s="111"/>
-      <c r="Q16" s="113"/>
-      <c r="R16" s="109"/>
+      <c r="N16" s="118"/>
+      <c r="O16" s="131"/>
+      <c r="P16" s="114"/>
+      <c r="Q16" s="116"/>
+      <c r="R16" s="112"/>
       <c r="S16" s="52"/>
     </row>
     <row r="17" spans="1:19" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2556,7 +2558,7 @@
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C17" s="126"/>
+      <c r="C17" s="129"/>
       <c r="D17" s="47" t="s">
         <v>18</v>
       </c>
@@ -2589,19 +2591,21 @@
         <v>500</v>
       </c>
       <c r="N17" s="62">
-        <v>510</v>
+        <v>35</v>
       </c>
       <c r="O17" s="83" t="s">
         <v>175</v>
       </c>
       <c r="P17" s="75">
-        <v>0.13200000000000001</v>
+        <v>1.8846153846153799</v>
       </c>
       <c r="Q17" s="56">
         <f t="shared" si="2"/>
-        <v>67.320000000000007</v>
-      </c>
-      <c r="R17" s="50"/>
+        <v>65.961538461538296</v>
+      </c>
+      <c r="R17" s="50" t="s">
+        <v>187</v>
+      </c>
       <c r="S17" s="51"/>
     </row>
     <row r="18" spans="1:19" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2610,7 +2614,7 @@
         <f>ROW(B18) - ROW($B$9)</f>
         <v>9</v>
       </c>
-      <c r="C18" s="124" t="s">
+      <c r="C18" s="127" t="s">
         <v>153</v>
       </c>
       <c r="D18" s="43" t="s">
@@ -2666,7 +2670,7 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="C19" s="125"/>
+      <c r="C19" s="128"/>
       <c r="D19" s="47" t="s">
         <v>20</v>
       </c>
@@ -2833,7 +2837,7 @@
         <f>ROW(B22) - ROW($B$9)</f>
         <v>13</v>
       </c>
-      <c r="C22" s="124" t="s">
+      <c r="C22" s="127" t="s">
         <v>155</v>
       </c>
       <c r="D22" s="43" t="s">
@@ -2889,7 +2893,7 @@
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="C23" s="125"/>
+      <c r="C23" s="128"/>
       <c r="D23" s="47" t="s">
         <v>24</v>
       </c>
@@ -2943,7 +2947,7 @@
         <f>ROW(B24) - ROW($B$9)</f>
         <v>15</v>
       </c>
-      <c r="C24" s="125"/>
+      <c r="C24" s="128"/>
       <c r="D24" s="43" t="s">
         <v>25</v>
       </c>
@@ -2997,7 +3001,7 @@
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="C25" s="125"/>
+      <c r="C25" s="128"/>
       <c r="D25" s="47" t="s">
         <v>26</v>
       </c>
@@ -3051,7 +3055,7 @@
         <f>ROW(B26) - ROW($B$9)</f>
         <v>17</v>
       </c>
-      <c r="C26" s="125"/>
+      <c r="C26" s="128"/>
       <c r="D26" s="43" t="s">
         <v>27</v>
       </c>
@@ -3105,7 +3109,7 @@
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="C27" s="125"/>
+      <c r="C27" s="128"/>
       <c r="D27" s="47" t="s">
         <v>28</v>
       </c>
@@ -3159,7 +3163,7 @@
         <f>ROW(B28) - ROW($B$9)</f>
         <v>19</v>
       </c>
-      <c r="C28" s="126"/>
+      <c r="C28" s="129"/>
       <c r="D28" s="43" t="s">
         <v>29</v>
       </c>
@@ -3326,7 +3330,7 @@
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
-      <c r="C31" s="125" t="s">
+      <c r="C31" s="128" t="s">
         <v>156</v>
       </c>
       <c r="D31" s="47" t="s">
@@ -3369,7 +3373,7 @@
         <v>137</v>
       </c>
       <c r="R31" s="79" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="S31" s="51"/>
     </row>
@@ -3379,7 +3383,7 @@
         <f>ROW(B32) - ROW($B$9)</f>
         <v>23</v>
       </c>
-      <c r="C32" s="125"/>
+      <c r="C32" s="128"/>
       <c r="D32" s="43" t="s">
         <v>33</v>
       </c>
@@ -3433,7 +3437,7 @@
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="C33" s="125"/>
+      <c r="C33" s="128"/>
       <c r="D33" s="47" t="s">
         <v>34</v>
       </c>
@@ -3487,7 +3491,7 @@
         <f>ROW(B34) - ROW($B$9)</f>
         <v>25</v>
       </c>
-      <c r="C34" s="125"/>
+      <c r="C34" s="128"/>
       <c r="D34" s="43" t="s">
         <v>35</v>
       </c>
@@ -3519,7 +3523,7 @@
         <v>505</v>
       </c>
       <c r="O34" s="100" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="P34" s="63">
         <v>2.29</v>
@@ -3529,7 +3533,7 @@
         <v>1156.45</v>
       </c>
       <c r="R34" s="84" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="S34" s="52"/>
     </row>
@@ -3539,7 +3543,7 @@
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
-      <c r="C35" s="124" t="s">
+      <c r="C35" s="127" t="s">
         <v>158</v>
       </c>
       <c r="D35" s="47" t="s">
@@ -3576,8 +3580,8 @@
       <c r="N35" s="62">
         <v>505</v>
       </c>
-      <c r="O35" s="130" t="s">
-        <v>185</v>
+      <c r="O35" s="106" t="s">
+        <v>184</v>
       </c>
       <c r="P35" s="75">
         <v>0.9</v>
@@ -3587,7 +3591,7 @@
         <v>454.5</v>
       </c>
       <c r="R35" s="79" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="S35" s="51"/>
     </row>
@@ -3597,7 +3601,7 @@
         <f>ROW(B36) - ROW($B$9)</f>
         <v>27</v>
       </c>
-      <c r="C36" s="126"/>
+      <c r="C36" s="129"/>
       <c r="D36" s="43" t="s">
         <v>37</v>
       </c>
@@ -3616,7 +3620,7 @@
       <c r="I36" s="61" t="s">
         <v>110</v>
       </c>
-      <c r="J36" s="131" t="s">
+      <c r="J36" s="107" t="s">
         <v>183</v>
       </c>
       <c r="K36" s="92" t="s">
@@ -3633,7 +3637,7 @@
         <v>510</v>
       </c>
       <c r="O36" s="100" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="P36" s="63">
         <v>0.44</v>
@@ -3643,7 +3647,7 @@
         <v>224.4</v>
       </c>
       <c r="R36" s="84" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="S36" s="53"/>
     </row>
@@ -3659,21 +3663,21 @@
       <c r="G37" s="37"/>
       <c r="H37" s="37"/>
       <c r="I37" s="36"/>
-      <c r="J37" s="132"/>
+      <c r="J37" s="108"/>
       <c r="K37" s="37"/>
       <c r="L37" s="37"/>
       <c r="M37" s="37"/>
-      <c r="N37" s="106" t="s">
+      <c r="N37" s="109" t="s">
         <v>179</v>
       </c>
-      <c r="O37" s="107"/>
-      <c r="P37" s="107"/>
+      <c r="O37" s="110"/>
+      <c r="P37" s="110"/>
       <c r="Q37" s="85">
         <f>SUM(Q10:Q36)</f>
-        <v>3036.6524999999997</v>
-      </c>
-      <c r="R37" s="120"/>
-      <c r="S37" s="121"/>
+        <v>3061.8940384615385</v>
+      </c>
+      <c r="R37" s="123"/>
+      <c r="S37" s="124"/>
     </row>
     <row r="38" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1"/>
@@ -3691,26 +3695,26 @@
       <c r="K38" s="10"/>
       <c r="L38" s="10"/>
       <c r="M38" s="10"/>
-      <c r="N38" s="106" t="s">
+      <c r="N38" s="109" t="s">
         <v>180</v>
       </c>
-      <c r="O38" s="107"/>
-      <c r="P38" s="129"/>
+      <c r="O38" s="110"/>
+      <c r="P38" s="132"/>
       <c r="Q38" s="86">
         <v>42.53</v>
       </c>
-      <c r="R38" s="122"/>
-      <c r="S38" s="123"/>
+      <c r="R38" s="125"/>
+      <c r="S38" s="126"/>
     </row>
     <row r="39" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="N39" s="106" t="s">
+      <c r="N39" s="109" t="s">
         <v>181</v>
       </c>
-      <c r="O39" s="107"/>
-      <c r="P39" s="107"/>
+      <c r="O39" s="110"/>
+      <c r="P39" s="110"/>
       <c r="Q39" s="87">
         <f>Q37/500</f>
-        <v>6.0733049999999995</v>
+        <v>6.123788076923077</v>
       </c>
     </row>
   </sheetData>
@@ -3790,26 +3794,26 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="O11" r:id="rId1" xr:uid="{C6B02148-4707-4901-B984-AFB9EF721279}"/>
-    <hyperlink ref="O14" r:id="rId2" xr:uid="{4B274F78-A9B9-473A-B0C3-8DFFB2910F7C}"/>
-    <hyperlink ref="O13" r:id="rId3" xr:uid="{C3C8F532-EF15-46A7-B5C6-DF3ED28BEDAE}"/>
-    <hyperlink ref="O10" r:id="rId4" xr:uid="{E7F1D38A-F6D7-49DD-AD8F-7D617BEA4FCB}"/>
-    <hyperlink ref="O12" r:id="rId5" xr:uid="{153D22AA-0C97-4F93-B9D8-44560DC0DB9B}"/>
-    <hyperlink ref="O22" r:id="rId6" xr:uid="{67D82A06-0E26-4D8A-BA1B-AA0997884CA8}"/>
-    <hyperlink ref="O24" r:id="rId7" xr:uid="{B2F39CEB-7408-448F-ABCE-10BA8C0C084B}"/>
-    <hyperlink ref="O23" r:id="rId8" xr:uid="{90644E0C-D9D3-4FBB-A6C9-F044DF99AA2C}"/>
-    <hyperlink ref="O25" r:id="rId9" xr:uid="{E13DDD7B-527B-4035-A117-0E8A528BCBC7}"/>
-    <hyperlink ref="O26" r:id="rId10" xr:uid="{EC77F680-C5DA-4773-BCCB-88AB1718A489}"/>
-    <hyperlink ref="O27" r:id="rId11" xr:uid="{815A3342-7A81-4389-9B49-94BA3C68A3E2}"/>
-    <hyperlink ref="O18" r:id="rId12" xr:uid="{ED3D1B58-94F7-4EA1-856F-4F1130EAE950}"/>
-    <hyperlink ref="O19" r:id="rId13" xr:uid="{7D994EC4-7BD4-4415-A0BB-1A8F4726EB2A}"/>
-    <hyperlink ref="O20" r:id="rId14" xr:uid="{F2AA434C-E8FC-4109-B38C-E3A167DFB339}"/>
-    <hyperlink ref="O30" r:id="rId15" xr:uid="{F25C6ACA-5304-4BBB-89FE-5C2F70CBCA87}"/>
-    <hyperlink ref="O32" r:id="rId16" xr:uid="{F0CEC956-9CBD-4081-9E02-541B43334ECA}"/>
-    <hyperlink ref="O33" r:id="rId17" xr:uid="{3D961140-2712-4F5B-B3F7-1A596F78428B}"/>
-    <hyperlink ref="O28" r:id="rId18" xr:uid="{E075B427-64F6-4177-AF2A-7BBE421C14A7}"/>
-    <hyperlink ref="O17" r:id="rId19" xr:uid="{33DB0923-3B38-405A-BBDD-6664383AF100}"/>
-    <hyperlink ref="O15" r:id="rId20" xr:uid="{35CE2201-5F33-4F0C-A2FA-23C8E510FC0B}"/>
+    <hyperlink ref="O11" r:id="rId1"/>
+    <hyperlink ref="O14" r:id="rId2"/>
+    <hyperlink ref="O13" r:id="rId3"/>
+    <hyperlink ref="O10" r:id="rId4"/>
+    <hyperlink ref="O12" r:id="rId5"/>
+    <hyperlink ref="O22" r:id="rId6"/>
+    <hyperlink ref="O24" r:id="rId7"/>
+    <hyperlink ref="O23" r:id="rId8"/>
+    <hyperlink ref="O25" r:id="rId9"/>
+    <hyperlink ref="O26" r:id="rId10"/>
+    <hyperlink ref="O27" r:id="rId11"/>
+    <hyperlink ref="O18" r:id="rId12"/>
+    <hyperlink ref="O19" r:id="rId13"/>
+    <hyperlink ref="O20" r:id="rId14"/>
+    <hyperlink ref="O30" r:id="rId15"/>
+    <hyperlink ref="O32" r:id="rId16"/>
+    <hyperlink ref="O33" r:id="rId17"/>
+    <hyperlink ref="O28" r:id="rId18"/>
+    <hyperlink ref="O17" r:id="rId19"/>
+    <hyperlink ref="O15" r:id="rId20"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId21"/>

</xml_diff>